<commit_message>
Track FPT outputs and add power-vs-RPM plot
</commit_message>
<xml_diff>
--- a/config_pipeline_fpt.xlsx
+++ b/config_pipeline_fpt.xlsx
@@ -692,7 +692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -737,6 +737,20 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>out_FPT e versionado neste repositorio; raw_FPT permanece fora do Git.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>O plot power_kw_vs_rpm.png faz parte do conjunto padrao de saidas.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>